<commit_message>
feat: complete 3-in-1 generator updates and workplace bullying manuals
</commit_message>
<xml_diff>
--- a/三合一單自動產生器/地點代號對照表.xlsx
+++ b/三合一單自動產生器/地點代號對照表.xlsx
@@ -4,12 +4,12 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" concurrentManualCount="8"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,10 +39,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>18P3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>EF180183B</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -56,6 +52,10 @@
   </si>
   <si>
     <t>12P7</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>18P3B</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -389,12 +389,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="14.375" customWidth="1"/>
+    <col min="1" max="2" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -402,15 +402,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -418,20 +418,20 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(3-in-1): fix transport notice append overwrite and 3-in-1 filename duplication by batch_no
</commit_message>
<xml_diff>
--- a/三合一單自動產生器/地點代號對照表.xlsx
+++ b/三合一單自動產生器/地點代號對照表.xlsx
@@ -39,10 +39,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>18P3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>EF180183B</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -56,6 +52,10 @@
   </si>
   <si>
     <t>12P7</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>18P3B</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -407,7 +407,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -420,18 +420,18 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
         <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>